<commit_message>
Updating student thesis titles, etc.
</commit_message>
<xml_diff>
--- a/CV.xlsx
+++ b/CV.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1438" uniqueCount="747">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1441" uniqueCount="749">
   <si>
     <t xml:space="preserve">degree</t>
   </si>
@@ -1920,6 +1920,12 @@
     <t xml:space="preserve">Harriet Mason</t>
   </si>
   <si>
+    <t xml:space="preserve">Visualising Uncertainty for Exploratory Data Analysis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Co-advised with Dianne Cook and Sarah Goodwin</t>
+  </si>
+  <si>
     <t xml:space="preserve">Economics</t>
   </si>
   <si>
@@ -1941,7 +1947,7 @@
     <t xml:space="preserve">UNL Undergraduate Research Program</t>
   </si>
   <si>
-    <t xml:space="preserve">Transferred to Southern Illinois University due to program elimination at UNL</t>
+    <t xml:space="preserve">Transferred to Southern Illinois University due to program elimination</t>
   </si>
   <si>
     <t xml:space="preserve">Student Name</t>
@@ -3796,13 +3802,19 @@
       <c r="F25" s="8" t="s">
         <v>625</v>
       </c>
+      <c r="G25" s="0" t="s">
+        <v>626</v>
+      </c>
+      <c r="H25" s="0" t="s">
+        <v>627</v>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="8" t="s">
         <v>579</v>
       </c>
       <c r="B26" s="8" t="s">
-        <v>626</v>
+        <v>628</v>
       </c>
       <c r="C26" s="12" t="s">
         <v>283</v>
@@ -3814,7 +3826,7 @@
         <v>2025</v>
       </c>
       <c r="F26" s="8" t="s">
-        <v>627</v>
+        <v>629</v>
       </c>
       <c r="G26" s="8" t="s">
         <v>623</v>
@@ -3828,7 +3840,7 @@
         <v>579</v>
       </c>
       <c r="B27" s="8" t="s">
-        <v>628</v>
+        <v>630</v>
       </c>
       <c r="C27" s="12" t="s">
         <v>283</v>
@@ -3840,7 +3852,7 @@
         <v>2025</v>
       </c>
       <c r="F27" s="8" t="s">
-        <v>629</v>
+        <v>631</v>
       </c>
       <c r="G27" s="8" t="s">
         <v>623</v>
@@ -3866,7 +3878,7 @@
         <v>2026</v>
       </c>
       <c r="F28" s="8" t="s">
-        <v>630</v>
+        <v>632</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3874,7 +3886,7 @@
         <v>579</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>626</v>
+        <v>628</v>
       </c>
       <c r="C29" s="12" t="s">
         <v>283</v>
@@ -3886,13 +3898,13 @@
         <v>2026</v>
       </c>
       <c r="F29" s="8" t="s">
-        <v>627</v>
+        <v>629</v>
       </c>
       <c r="G29" s="8" t="s">
-        <v>631</v>
+        <v>633</v>
       </c>
       <c r="H29" s="1" t="s">
-        <v>632</v>
+        <v>634</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3914,8 +3926,11 @@
       <c r="F30" s="0" t="s">
         <v>624</v>
       </c>
+      <c r="G30" s="0" t="s">
+        <v>393</v>
+      </c>
       <c r="H30" s="0" t="s">
-        <v>633</v>
+        <v>635</v>
       </c>
     </row>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -3940,16 +3955,16 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>634</v>
+        <v>636</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>322</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>635</v>
+        <v>637</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>636</v>
+        <v>638</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>18</v>
@@ -3957,16 +3972,16 @@
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>637</v>
+        <v>639</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>638</v>
+        <v>640</v>
       </c>
       <c r="C2" s="4" t="n">
         <v>45007</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>639</v>
+        <v>641</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>12</v>
@@ -3974,7 +3989,7 @@
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>640</v>
+        <v>642</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>14</v>
@@ -3991,7 +4006,7 @@
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>641</v>
+        <v>643</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>14</v>
@@ -4000,7 +4015,7 @@
         <v>44774</v>
       </c>
       <c r="D4" s="13" t="s">
-        <v>642</v>
+        <v>644</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>16</v>
@@ -4008,7 +4023,7 @@
     </row>
     <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>643</v>
+        <v>645</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>14</v>
@@ -4025,7 +4040,7 @@
     </row>
     <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>644</v>
+        <v>646</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>14</v>
@@ -4034,7 +4049,7 @@
         <v>44409</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>639</v>
+        <v>641</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>16</v>
@@ -4042,13 +4057,13 @@
     </row>
     <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>645</v>
+        <v>647</v>
       </c>
       <c r="B7" s="8" t="s">
         <v>14</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>646</v>
+        <v>648</v>
       </c>
       <c r="E7" s="8" t="s">
         <v>16</v>
@@ -4090,10 +4105,10 @@
         <v>36</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>647</v>
+        <v>649</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>648</v>
+        <v>650</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>144</v>
@@ -4101,7 +4116,7 @@
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>649</v>
+        <v>651</v>
       </c>
       <c r="B2" s="1" t="b">
         <f aca="false">TRUE()</f>
@@ -4114,18 +4129,18 @@
         <v>2019</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>650</v>
+        <v>652</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>208</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>651</v>
+        <v>653</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>649</v>
+        <v>651</v>
       </c>
       <c r="B3" s="1" t="b">
         <f aca="false">TRUE()</f>
@@ -4138,18 +4153,18 @@
         <v>2021</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>652</v>
+        <v>654</v>
       </c>
       <c r="F3" s="1" t="s">
+        <v>655</v>
+      </c>
+      <c r="G3" s="1" t="s">
         <v>653</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>651</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>649</v>
+        <v>651</v>
       </c>
       <c r="B4" s="1" t="b">
         <f aca="false">FALSE()</f>
@@ -4162,16 +4177,16 @@
         <v>2019</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>654</v>
+        <v>656</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>655</v>
+        <v>657</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>656</v>
+        <v>658</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>657</v>
+        <v>659</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4189,21 +4204,21 @@
         <v>2020</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>652</v>
+        <v>654</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>658</v>
+        <v>660</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>659</v>
+        <v>661</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>660</v>
+        <v>662</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>649</v>
+        <v>651</v>
       </c>
       <c r="B6" s="1" t="b">
         <f aca="false">TRUE()</f>
@@ -4216,15 +4231,15 @@
         <v>2026</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>661</v>
+        <v>663</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>662</v>
+        <v>664</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>649</v>
+        <v>651</v>
       </c>
       <c r="B7" s="1" t="b">
         <f aca="false">TRUE()</f>
@@ -4237,18 +4252,18 @@
         <v>2022</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>663</v>
+        <v>665</v>
       </c>
       <c r="F7" s="1" t="s">
         <v>208</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>651</v>
+        <v>653</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>649</v>
+        <v>651</v>
       </c>
       <c r="B8" s="1" t="b">
         <f aca="false">TRUE()</f>
@@ -4261,10 +4276,10 @@
         <v>2020</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>664</v>
+        <v>666</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>665</v>
+        <v>667</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4285,15 +4300,15 @@
         <v>560</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>666</v>
+        <v>668</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>659</v>
+        <v>661</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>667</v>
+        <v>669</v>
       </c>
       <c r="B10" s="1" t="b">
         <f aca="false">FALSE()</f>
@@ -4306,18 +4321,18 @@
         <v>2020</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>668</v>
+        <v>670</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>669</v>
+        <v>671</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>670</v>
+        <v>672</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>649</v>
+        <v>651</v>
       </c>
       <c r="B11" s="1" t="b">
         <f aca="false">TRUE()</f>
@@ -4330,15 +4345,15 @@
         <v>2024</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>661</v>
+        <v>663</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>671</v>
+        <v>673</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>667</v>
+        <v>669</v>
       </c>
       <c r="B12" s="1" t="b">
         <f aca="false">TRUE()</f>
@@ -4351,21 +4366,21 @@
         <v>2025</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>672</v>
+        <v>674</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>673</v>
+        <v>675</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>674</v>
+        <v>676</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>675</v>
+        <v>677</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>667</v>
+        <v>669</v>
       </c>
       <c r="B13" s="1" t="b">
         <f aca="false">TRUE()</f>
@@ -4378,13 +4393,13 @@
         <v>2022</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>676</v>
+        <v>678</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>677</v>
+        <v>679</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>678</v>
+        <v>680</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4402,15 +4417,15 @@
         <v>2022</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>652</v>
+        <v>654</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>679</v>
+        <v>681</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>667</v>
+        <v>669</v>
       </c>
       <c r="B15" s="1" t="b">
         <f aca="false">FALSE()</f>
@@ -4423,15 +4438,15 @@
         <v>2021</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>652</v>
+        <v>654</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>680</v>
+        <v>682</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>667</v>
+        <v>669</v>
       </c>
       <c r="B16" s="1" t="b">
         <f aca="false">FALSE()</f>
@@ -4444,18 +4459,18 @@
         <v>2021</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>652</v>
+        <v>654</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>681</v>
+        <v>683</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>682</v>
+        <v>684</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>649</v>
+        <v>651</v>
       </c>
       <c r="B17" s="1" t="b">
         <f aca="false">TRUE()</f>
@@ -4468,18 +4483,18 @@
         <v>2023</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>683</v>
+        <v>685</v>
       </c>
       <c r="F17" s="1" t="s">
         <v>208</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>651</v>
+        <v>653</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>667</v>
+        <v>669</v>
       </c>
       <c r="B18" s="1" t="b">
         <f aca="false">TRUE()</f>
@@ -4492,18 +4507,18 @@
         <v>2026</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>684</v>
+        <v>686</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>659</v>
+        <v>661</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>685</v>
+        <v>687</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>649</v>
+        <v>651</v>
       </c>
       <c r="B19" s="1" t="b">
         <f aca="false">TRUE()</f>
@@ -4516,18 +4531,18 @@
         <v>2025</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>652</v>
+        <v>654</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>686</v>
+        <v>688</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>651</v>
+        <v>653</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>649</v>
+        <v>651</v>
       </c>
       <c r="B20" s="1" t="b">
         <f aca="false">TRUE()</f>
@@ -4540,18 +4555,18 @@
         <v>2024</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>687</v>
+        <v>689</v>
       </c>
       <c r="F20" s="1" t="s">
         <v>208</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>651</v>
+        <v>653</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>667</v>
+        <v>669</v>
       </c>
       <c r="B21" s="1" t="b">
         <f aca="false">TRUE()</f>
@@ -4564,18 +4579,18 @@
         <v>2024</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>652</v>
+        <v>654</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>688</v>
+        <v>690</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>685</v>
+        <v>687</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>667</v>
+        <v>669</v>
       </c>
       <c r="B22" s="1" t="b">
         <f aca="false">TRUE()</f>
@@ -4588,21 +4603,21 @@
         <v>2026</v>
       </c>
       <c r="E22" s="8" t="s">
-        <v>652</v>
+        <v>654</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>685</v>
+        <v>687</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>689</v>
+        <v>691</v>
       </c>
       <c r="H22" s="8" t="s">
-        <v>690</v>
+        <v>692</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="8" t="s">
-        <v>649</v>
+        <v>651</v>
       </c>
       <c r="B23" s="7" t="n">
         <f aca="false">TRUE()</f>
@@ -4618,13 +4633,13 @@
         <v>560</v>
       </c>
       <c r="F23" s="8" t="s">
-        <v>691</v>
+        <v>693</v>
       </c>
       <c r="G23" s="8" t="s">
-        <v>692</v>
+        <v>694</v>
       </c>
       <c r="H23" s="8" t="s">
-        <v>693</v>
+        <v>695</v>
       </c>
     </row>
   </sheetData>
@@ -4651,7 +4666,7 @@
         <v>510</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>694</v>
+        <v>696</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4659,7 +4674,7 @@
         <v>2022</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>671</v>
+        <v>673</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4667,7 +4682,7 @@
         <v>2019</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>662</v>
+        <v>664</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4675,7 +4690,7 @@
         <v>2020</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>695</v>
+        <v>697</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4683,7 +4698,7 @@
         <v>2020</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>696</v>
+        <v>698</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4691,7 +4706,7 @@
         <v>2020</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>697</v>
+        <v>699</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4699,7 +4714,7 @@
         <v>2021</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>698</v>
+        <v>700</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4707,7 +4722,7 @@
         <v>2021</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>699</v>
+        <v>701</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4715,7 +4730,7 @@
         <v>2021</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>700</v>
+        <v>702</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4723,7 +4738,7 @@
         <v>2022</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>701</v>
+        <v>703</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4731,7 +4746,7 @@
         <v>2020</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>702</v>
+        <v>704</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4739,7 +4754,7 @@
         <v>2021</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>702</v>
+        <v>704</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4747,7 +4762,7 @@
         <v>2022</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>702</v>
+        <v>704</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4755,7 +4770,7 @@
         <v>2023</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>702</v>
+        <v>704</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4763,7 +4778,7 @@
         <v>2022</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>698</v>
+        <v>700</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4771,7 +4786,7 @@
         <v>2023</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>671</v>
+        <v>673</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4779,7 +4794,7 @@
         <v>2023</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>703</v>
+        <v>705</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4787,7 +4802,7 @@
         <v>2023</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>662</v>
+        <v>664</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4795,7 +4810,7 @@
         <v>2023</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>671</v>
+        <v>673</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4803,7 +4818,7 @@
         <v>2025</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>698</v>
+        <v>700</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4811,7 +4826,7 @@
         <v>2025</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>704</v>
+        <v>706</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4819,7 +4834,7 @@
         <v>2025</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>662</v>
+        <v>664</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4827,7 +4842,7 @@
         <v>2025</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>703</v>
+        <v>705</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4835,7 +4850,7 @@
         <v>2026</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>705</v>
+        <v>707</v>
       </c>
     </row>
   </sheetData>
@@ -4862,22 +4877,22 @@
         <v>1</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>706</v>
+        <v>708</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>707</v>
+        <v>709</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>144</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>709</v>
+        <v>711</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>710</v>
+        <v>712</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4892,10 +4907,10 @@
         <v>2023</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>711</v>
+        <v>713</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>712</v>
+        <v>714</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4910,10 +4925,10 @@
         <v>2023</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>713</v>
+        <v>715</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>714</v>
+        <v>716</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4928,10 +4943,10 @@
         <v>2022</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>715</v>
+        <v>717</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>716</v>
+        <v>718</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4946,7 +4961,7 @@
         <v>2020</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>717</v>
+        <v>719</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4961,10 +4976,10 @@
         <v>2020</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>718</v>
+        <v>720</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>719</v>
+        <v>721</v>
       </c>
     </row>
   </sheetData>
@@ -5000,10 +5015,10 @@
         <v>35</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>706</v>
+        <v>708</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>707</v>
+        <v>709</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>144</v>
@@ -5012,13 +5027,13 @@
         <v>38</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>709</v>
+        <v>711</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>710</v>
+        <v>712</v>
       </c>
       <c r="J1" s="1"/>
       <c r="K1" s="1"/>
@@ -5030,7 +5045,7 @@
         <v>0</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>720</v>
+        <v>722</v>
       </c>
       <c r="C2" s="1" t="n">
         <v>2025</v>
@@ -5039,13 +5054,13 @@
         <v>2025</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>721</v>
+        <v>723</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>722</v>
+        <v>724</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>723</v>
+        <v>725</v>
       </c>
       <c r="H2" s="1"/>
       <c r="I2" s="1"/>
@@ -5059,7 +5074,7 @@
         <v>0</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>720</v>
+        <v>722</v>
       </c>
       <c r="C3" s="1" t="n">
         <v>2025</v>
@@ -5068,13 +5083,13 @@
         <v>2026</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>724</v>
+        <v>726</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>725</v>
+        <v>727</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>726</v>
+        <v>728</v>
       </c>
       <c r="H3" s="1"/>
       <c r="I3" s="1"/>
@@ -5088,7 +5103,7 @@
         <v>0</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>720</v>
+        <v>722</v>
       </c>
       <c r="C4" s="1" t="n">
         <v>2025</v>
@@ -5097,13 +5112,13 @@
         <v>2026</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>724</v>
+        <v>726</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>727</v>
+        <v>729</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>728</v>
+        <v>730</v>
       </c>
       <c r="H4" s="1"/>
       <c r="I4" s="1"/>
@@ -5117,7 +5132,7 @@
         <v>0</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>720</v>
+        <v>722</v>
       </c>
       <c r="C5" s="1" t="n">
         <v>2024</v>
@@ -5126,13 +5141,13 @@
         <v>2025</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>721</v>
+        <v>723</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>727</v>
+        <v>729</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>729</v>
+        <v>731</v>
       </c>
       <c r="H5" s="1"/>
       <c r="I5" s="1"/>
@@ -5146,7 +5161,7 @@
         <v>0</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>720</v>
+        <v>722</v>
       </c>
       <c r="C6" s="9" t="n">
         <v>2023</v>
@@ -5155,13 +5170,13 @@
         <v>2023</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>721</v>
+        <v>723</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>731</v>
+        <v>733</v>
       </c>
       <c r="I6" s="1"/>
       <c r="J6" s="1"/>
@@ -5174,7 +5189,7 @@
         <v>0</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>720</v>
+        <v>722</v>
       </c>
       <c r="C7" s="9" t="n">
         <v>2022</v>
@@ -5183,13 +5198,13 @@
         <v>2022</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>721</v>
+        <v>723</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>732</v>
+        <v>734</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>733</v>
+        <v>735</v>
       </c>
       <c r="I7" s="1"/>
       <c r="J7" s="1"/>
@@ -5202,7 +5217,7 @@
         <v>0</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>720</v>
+        <v>722</v>
       </c>
       <c r="C8" s="9" t="n">
         <v>2022</v>
@@ -5211,13 +5226,13 @@
         <v>2022</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>721</v>
+        <v>723</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>734</v>
+        <v>736</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>735</v>
+        <v>737</v>
       </c>
       <c r="I8" s="1"/>
       <c r="J8" s="1"/>
@@ -5230,7 +5245,7 @@
         <v>0</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>720</v>
+        <v>722</v>
       </c>
       <c r="C9" s="9" t="n">
         <v>2022</v>
@@ -5239,13 +5254,13 @@
         <v>2022</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>721</v>
+        <v>723</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>736</v>
+        <v>738</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>737</v>
+        <v>739</v>
       </c>
       <c r="I9" s="1"/>
       <c r="J9" s="1"/>
@@ -5258,7 +5273,7 @@
         <v>0</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>720</v>
+        <v>722</v>
       </c>
       <c r="C10" s="9" t="n">
         <v>2021</v>
@@ -5267,13 +5282,13 @@
         <v>2021</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>721</v>
+        <v>723</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>736</v>
+        <v>738</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>738</v>
+        <v>740</v>
       </c>
       <c r="H10" s="1"/>
       <c r="I10" s="1"/>
@@ -5287,7 +5302,7 @@
         <v>0</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>739</v>
+        <v>741</v>
       </c>
       <c r="C11" s="9" t="n">
         <v>2021</v>
@@ -5296,13 +5311,13 @@
         <v>2021</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>740</v>
+        <v>742</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>741</v>
+        <v>743</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>742</v>
+        <v>744</v>
       </c>
       <c r="H11" s="1"/>
       <c r="I11" s="1"/>
@@ -5316,7 +5331,7 @@
         <v>0</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>739</v>
+        <v>741</v>
       </c>
       <c r="C12" s="9" t="n">
         <v>2021</v>
@@ -5328,10 +5343,10 @@
         <v>352</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>741</v>
+        <v>743</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>743</v>
+        <v>745</v>
       </c>
       <c r="H12" s="1"/>
       <c r="I12" s="1"/>
@@ -5345,7 +5360,7 @@
         <v>0</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>739</v>
+        <v>741</v>
       </c>
       <c r="C13" s="9" t="n">
         <v>2020</v>
@@ -5354,16 +5369,16 @@
         <v>2020</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>744</v>
+        <v>746</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>741</v>
+        <v>743</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>745</v>
+        <v>747</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>746</v>
+        <v>748</v>
       </c>
       <c r="I13" s="1"/>
       <c r="J13" s="1"/>

</xml_diff>